<commit_message>
Add 2,110 test cases across 5 domains (400+ each, ~96.5% pass rate) with interactive report link
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Execution_Summary.xlsx
+++ b/Test Results/Excel/Execution_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1425</v>
+        <v>2110</v>
       </c>
     </row>
     <row r="3">
@@ -464,7 +464,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1416</v>
+        <v>2036</v>
       </c>
     </row>
     <row r="4">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5">
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -495,7 +495,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>99.37%</t>
+          <t>96.49%</t>
         </is>
       </c>
     </row>

</xml_diff>